<commit_message>
added howard county to zoning workbook
</commit_message>
<xml_diff>
--- a/Zoning_Workbook.xlsx
+++ b/Zoning_Workbook.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/055abc5dbe1424b0/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="8_{8AA4DF28-16B8-4606-B3D8-82A740A57BE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AF6802ED-8996-4507-9322-4782E8AB9907}"/>
+  <xr:revisionPtr revIDLastSave="254" documentId="8_{8AA4DF28-16B8-4606-B3D8-82A740A57BE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C68759DE-1CC9-43D9-A3C8-F50A309ABA09}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3F8FDE9A-8AA9-43D2-80E0-CEBDCEE92368}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3F8FDE9A-8AA9-43D2-80E0-CEBDCEE92368}"/>
   </bookViews>
   <sheets>
     <sheet name="Frederick County" sheetId="1" r:id="rId1"/>
@@ -18,8 +18,9 @@
     <sheet name="Allegany County" sheetId="3" r:id="rId3"/>
     <sheet name="Montgomery County" sheetId="4" r:id="rId4"/>
     <sheet name="Garrett County" sheetId="5" r:id="rId5"/>
+    <sheet name="Howard County" sheetId="6" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="191029" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="331">
   <si>
     <t>Zone</t>
   </si>
@@ -910,12 +911,318 @@
   <si>
     <t>The purpose of the Resource Conservation Zoning District is to allow low intensity uses and activities which are compatible with the goal of resource conservation to be located within mountain and rural wooded areas. Areas within this district include mountain areas, rural woodlands, and cultural, scenic, and recreation resource areas. Environmentally sensitive areas within the resource conservation zone, including FEMA floodplain, steep slopes, wetlands and the habitats of threatened and endangered species, will be protected from development.</t>
   </si>
+  <si>
+    <t>Rural Conservation</t>
+  </si>
+  <si>
+    <t>Howard County Planning and Zoning Department</t>
+  </si>
+  <si>
+    <t>The Rural Conservation District is established to conserve farmland and to encourage agricultural activities, thereby helping to ensure that commercial agriculture will continue as a long term land use and a viable economic activity within the County. The RC District is also established to preserve natural features and the rural landscape, while allowing low density, clustered residential development. Residential development is to be permitted only when it is located and designed to minimize its impact on agricultural land, farming operations, and sensitive environmental features; to create attractive rural developments; and to respect existing features of the rural landscape.</t>
+  </si>
+  <si>
+    <t>Rural Residential</t>
+  </si>
+  <si>
+    <t>The Rural Residential District is established to allow low density residential development within a rural environment. The Rural Residential District is intended for an area of the County which is already largely committed to low density residential subdivisions. Within the RR District, agriculture is permitted as well as residential development in both cluster and non-cluster forms. Cluster development is permitted in order to protect environmental and landscape resources and to preserve agricultural land.</t>
+  </si>
+  <si>
+    <t>Density Exchange Option</t>
+  </si>
+  <si>
+    <t>DEO</t>
+  </si>
+  <si>
+    <t>The DEO Overlay District is established to provide land owners in the RC and RR Districts with opportunity and incentive to preserve significant blocks of farmland in the rural area of the county. This district is also intended to encourage the clustering of residential development in areas where the development will not have an adverse impact on farm operations. To accomplish this, the DEO District allows residential density in the RC and RR Districts to be exchanged between parcels. Density exchanges in the District should result in large parcels being preserved in perpetuity, while residential development is directed toward parcels which are able to absorb the additional dwellings.</t>
+  </si>
+  <si>
+    <t>Residential: Environmental Development</t>
+  </si>
+  <si>
+    <t>R-ED</t>
+  </si>
+  <si>
+    <t>The R-ED District is established to accommodate residential development at a density of two dwelling units per net acre in areas with a high proportion of sensitive environmental and/or historic resources. Protection of environmental and historic resources is to be achieved by minimizing the amount of site disturbance and directing development to the most appropriate areas of a site, away from sensitive resources. To accomplish this, the regulations allow site planning flexibility and require that development proposals be evaluated in terms of their effectiveness in minimizing alteration of existing topography, vegetation and the landscape setting for historic structures.</t>
+  </si>
+  <si>
+    <t>Residential: Single</t>
+  </si>
+  <si>
+    <t>The R-20 District is established to permit single-family detached dwelling units at approximately two units per acre. The District reflects the established single-family neighborhood characteristics of many of the stable residential areas of the county.</t>
+  </si>
+  <si>
+    <t>The R-12 District is established to provide single-family detached and semi-detached residential uses. The district provides a choice of housing types typically on lots less than a half acre.</t>
+  </si>
+  <si>
+    <t>R-SC</t>
+  </si>
+  <si>
+    <t>Residential: Single Cluster</t>
+  </si>
+  <si>
+    <t>The R-SC District is established to provide the opportunity for clustering of single-family detached and attached dwellings to promote sensitive use for the land as well as to provide compatibility with other residential districts.</t>
+  </si>
+  <si>
+    <t>R-SA-8</t>
+  </si>
+  <si>
+    <t>Residential: Single Attached</t>
+  </si>
+  <si>
+    <t>The R-SA-8 District is established to provide clustered attached dwelling units. It is the intent of this district that the attached dwellings be compatible with adjacent residential zones.</t>
+  </si>
+  <si>
+    <t>Residential: Historic - Environmental District</t>
+  </si>
+  <si>
+    <t>R-H-ED</t>
+  </si>
+  <si>
+    <t>The R-H-ED District is established to provide requirements for single-family attached dwelling units on certain properties determined to contribute to the historic character of areas designated on the National Register of Historic Places. It is the intent of this district that the attached dwellings be compatible with the historic character of the area, and be developed with sensitivity to the natural environment. Protection of historic and environmental resources is to be achieved by requiring Historic District Commission review and directing development away from sensitive resources.</t>
+  </si>
+  <si>
+    <t>R-APT</t>
+  </si>
+  <si>
+    <t>Residential: Apartments</t>
+  </si>
+  <si>
+    <t>The R-APT district is established to provide the opportunity for higher density apartments to support adjacent retail areas and services, enhance transportation hubs and provide a land use transition between more intense uses and lower density residential districts. It is intended that R-APT districts will adjoin arterial roadways and should have opportunities for pedestrian and bicycle access to the surrounding areas.</t>
+  </si>
+  <si>
+    <t>R-MH</t>
+  </si>
+  <si>
+    <t>Residential: Mobile Home</t>
+  </si>
+  <si>
+    <t>The R-MH District is established to provide the opportunity for moderately priced housing. It is the intent of the district that opportunities for home ownership and rental sites be maintained.</t>
+  </si>
+  <si>
+    <t>Residential: Senior - Institutional</t>
+  </si>
+  <si>
+    <t>R-SI</t>
+  </si>
+  <si>
+    <t>The Residential: Senior—Institutional (R-SI) District is established to permit age-restricted adult housing, as well as community-serving institutional and cultural facilities that serve the surrounding residential community.</t>
+  </si>
+  <si>
+    <t>Institutional</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t>The Institutional District (I) is established to permit community-serving institutional and cultural facilities. These uses benefit the surrounding residential community and may in some locations provide a transition between residential neighborhoods and retail activity centers. The Institutional District is an Overlay District. Uses allowed in the underlying district may be established prior to approval of a Preliminary Development Plan for institutional district development.</t>
+  </si>
+  <si>
+    <t>Residential: Village Housing</t>
+  </si>
+  <si>
+    <t>R-VH</t>
+  </si>
+  <si>
+    <t>The R-VH District is established to permit infill development compatible with the historic lot patterns within an Historic District. The district is intended to encourage the use and redevelopment of residential enclaves consistent with the character of existing development.</t>
+  </si>
+  <si>
+    <t>Historic: Office</t>
+  </si>
+  <si>
+    <t>HO</t>
+  </si>
+  <si>
+    <t>The Historic Office District is established to permit a mix of offices and residences with supporting cultural and commercial uses which will encourage new development and reuse of existing structures consistent with the existing character of the area.</t>
+  </si>
+  <si>
+    <t>Historic: Commercial</t>
+  </si>
+  <si>
+    <t>HC</t>
+  </si>
+  <si>
+    <t>The Historic Commercial District is established to permit and encourage a diverse but compatible and complementary mix of commercial, office, cultural and residential activities. The district is intended to encourage development of a pedestrian environment consistent with the overall development concept for the Historic District.</t>
+  </si>
+  <si>
+    <t>Planned Office Research</t>
+  </si>
+  <si>
+    <t>POR</t>
+  </si>
+  <si>
+    <t>The Planned Office Research District is established to permit and encourage diverse institutional, commercial, office research and cultural facilities.</t>
+  </si>
+  <si>
+    <t>Planned Employment Center</t>
+  </si>
+  <si>
+    <t>PEC</t>
+  </si>
+  <si>
+    <t>The PEC District is established to provide for comprehensively planned employment centers combining research and development, office, light manufacturing and assembly, limited commercial and other enumerated uses. It is intended that this district provide higher standards of development and a more flexible approach to design and development than could be achieved under conventional zoning districts. It is further the purpose of this district to: Provide for orderly development of large-scale, comprehensively planned employment centers; Provide for open areas to act as buffers between incompatible uses and as design elements which will achieve the physical and aesthetic integration of the uses and activities within each development; and Provide a landscaped, campus-like setting for employment in which the various uses relate compatibly with one another according to a comprehensive plan of development for an entire district.</t>
+  </si>
+  <si>
+    <t>Business: Rural</t>
+  </si>
+  <si>
+    <t>BR</t>
+  </si>
+  <si>
+    <t>The BR District is established to allow the development of businesses which will support the agricultural industry, serve the needs of the rural residential and farming communities, and provide opportunity for a combination of business and industrial uses not otherwise permitted in the rural areas of the County. Appropriate locations for the land uses allowed in the BR District depend on factors, which are best examined through review of a particular site. Therefore, the BR District is a floating zone, which requires the submission of a Preliminary Development Plan for a particular site. It is intended that the BR District be applied at a particular location only if found to be appropriate with respect to road access and compatibility with neighboring land uses.</t>
+  </si>
+  <si>
+    <t>Office Trasition</t>
+  </si>
+  <si>
+    <t>OT</t>
+  </si>
+  <si>
+    <t>The OT District is established to allow office and other low-intensity commercial uses adjacent to areas of residential zoning. The OT District is a floating district that will provide a transition along the edges of residential areas impacted by arterial highways carrying high volumes of traffic. The standards of this district should result in small-scale commercial buildings on attractively-designed sites that are compatible with neighboring residential uses.</t>
+  </si>
+  <si>
+    <t>CCT</t>
+  </si>
+  <si>
+    <t>Community Center Transition</t>
+  </si>
+  <si>
+    <t>The CCT (Community Center Transition) District is established to permit community serving office, institutional, service and cultural facilities, as well as age-restricted adult housing. These uses serve the community and provide a transition between residential neighborhoods and non-residential development or an arterial highway.</t>
+  </si>
+  <si>
+    <t>Business: Local</t>
+  </si>
+  <si>
+    <t>The B-1 District is established to provide areas of local business that can directly serve the general public with retail sales and services.</t>
+  </si>
+  <si>
+    <t>B-2</t>
+  </si>
+  <si>
+    <t>The B-2 District is established to provide for commercial sales and services that directly serve the general public.</t>
+  </si>
+  <si>
+    <t>Business: General</t>
+  </si>
+  <si>
+    <t>Shoppig Center</t>
+  </si>
+  <si>
+    <t>SC</t>
+  </si>
+  <si>
+    <t>The SC District is established to permit local retail and office use areas. The Shopping Center District permits the opportunity for one stop shopping for a neighborhood and community.</t>
+  </si>
+  <si>
+    <t>Community Enhancement Floating</t>
+  </si>
+  <si>
+    <t>CEF</t>
+  </si>
+  <si>
+    <t>The Community Enhancement Floating (CEF) District is established to encourage the creative development and redevelopment of commercial and residential properties through flexible zoning so that the proposed development complements and enhances the surrounding uses and creates a more coherent, connected development. While it is envisioned that the CEF District could place residential uses on land zoned for employment in some circumstances, it should not be viewed primarily as a way to convert land zoned for employment to residential.</t>
+  </si>
+  <si>
+    <t>Manufacturing: Light</t>
+  </si>
+  <si>
+    <t>M-1</t>
+  </si>
+  <si>
+    <t>The M-1 District is established to permit a mix of manufacturing, warehousing and business uses with provisions for limited retail sales.</t>
+  </si>
+  <si>
+    <t>Manufacturing: Heavy</t>
+  </si>
+  <si>
+    <t>M-2</t>
+  </si>
+  <si>
+    <t>The M-2 District is established to permit a mix of manufacturing, warehousing, industrial and business uses with provisions for limited retail sales.</t>
+  </si>
+  <si>
+    <t>Solid Waste</t>
+  </si>
+  <si>
+    <t>SW</t>
+  </si>
+  <si>
+    <t>The Solid Waste District is established to provide opportunity for solid waste processing facilities not allowed in other zoning districts and to encourage re-use and recycling of solid waste in lieu of disposal at a landfill. Because of changing technology, it is not possible to identify and adopt specific Zoning Regulations for all types of solid waste processing uses which may be proposed in Howard County. However, it is essential to provide opportunity for viable, constructive alternatives to disposal of solid waste in landfills. The Solid Waste District permits processing facilities for non-hazardous solid waste which are not covered elsewhere in the Zoning Regulations, while requiring detailed review of each proposal to evaluate its land use impacts and its potential contribution to the County's solid waste management system. Because many solid waste processing facilities are of a heavy industrial nature, the SW District is an overlay district which may be applied only to land in the M-2 District. The Zoning Board may also apply the SW District to land in the M-1 District, provided there is a compelling reason and the use in the SW District shall be limited to a waste transfer station or material recovery facility. The SW District is a floating district which may be applied if the Zoning Board finds, upon review of a specific proposal and Preliminary Development Plan, that application of the District at a proposed location will meet the requirements established in this Section.</t>
+  </si>
+  <si>
+    <t>Planned Golf Course Community</t>
+  </si>
+  <si>
+    <t>PGCC</t>
+  </si>
+  <si>
+    <t>The Planned Golf Course Community District is established to permit mixed use development combining recreation, residential, commercial and conference center uses while preserving 50% of the district as open space. It is the purpose of the PGCC District to integrate recreational uses, including at least two eighteen-hole golf courses, with residential development and to provide a variety of housing choices.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mixed Use </t>
+  </si>
+  <si>
+    <t>MXD</t>
+  </si>
+  <si>
+    <t>The Mixed Use Districts are established to permit flexible and efficient use of large parcels at key locations by combining housing, employment, local commercial and open space uses in accordance with a unified design. Appropriate locations for the MXD Districts will be characterized by availability of public utilities, good access to collector or arterial highways, and potential access to public transit facilities. The phasing of development in the MXD Districts is to be concurrent with the phasing of required road improvements and is to result in a mix of land uses at the earliest feasible stage of development. The MXD Districts provide for well-designed communities which are compatible with surrounding neighborhoods and protective of the natural elements of the landscape. A Mixed Use Development is intended to include a planned network of open space which includes environmental areas, recreation areas, and public plazas or squares; a diversity of housing types at medium to high densities; and convenient pedestrian access between uses. Two MXD Districts are established: the MXD-3 and MXD-6 Districts. The two districts allow differing intensities of land use in order to ensure that mixed use developments are compatible with surrounding land uses. A Mixed Use Development shall contain at least one focal point: an area of diverse, integrated land uses, designed to create a distinct focus for the development. Focal points should be scaled and oriented to pedestrian movement and should incorporate public transit access if available. The MXD District regulations promote and allow planning innovation and design flexibility. Each plan submission for an MXD District must incorporate design considerations at an appropriate level of detail for the submission stage. A public hearing is required at the Preliminary Development Plan and Comprehensive Sketch Plan stages of the plan review process, to ensure adequate opportunity for public comment. In order to allow appropriate uses prior to the approval of a Mixed Use Development, the MXD-3 and MXD-6 Districts are Overlay Districts. Uses allowed in the underlying district may be established prior to the approval of a Preliminary Development Plan for Mixed Use Development.</t>
+  </si>
+  <si>
+    <t>Planned Senior Community</t>
+  </si>
+  <si>
+    <t>PSC</t>
+  </si>
+  <si>
+    <t>The Planned Senior Community District is established to permit the development of housing designed for older adults and elderly persons. This floating and overlay district provides opportunity for housing that meets the diverse needs of Howard County's growing senior population. Each Planned Senior Community District will provide independent living units for seniors within either single-family or multi-family dwellings, and may also include assisted living or nursing care facilities. The communities developed within the PSC District will be characterized by careful site planning that allows them to be compatible with eastern Howard County's residential neighborhoods.</t>
+  </si>
+  <si>
+    <t>Corridor Employment</t>
+  </si>
+  <si>
+    <t>The CE District is intended to encourage the development and redevelopment of employment land near U.S. Route 1. Development in the CE District should provide for new office, flex, and light industrial uses, while reducing the spread of strip commercial development and encouraging consolidation of fragmented parcels. The requirements of this district, in conjunction with the Route 1 Manual and required vehicular and pedestrian improvements, will result in development that improves the appearance of the Route 1 streetscape, enhances traffic safety and better accommodates public transit and pedestrian travel. Many parcels in the CE District were developed before this district was created. It is not the intent of these requirements to disallow the continued use of sites developed prior to the CE District. The intent of this district will be achieved by bringing sites into compliance with these requirements and the standards of the Route 1 Manual as uses are redeveloped or expanded.</t>
+  </si>
+  <si>
+    <t>Continuing Light Industrial</t>
+  </si>
+  <si>
+    <t>CLI</t>
+  </si>
+  <si>
+    <t>The Continuing Light Industrial (CLI) Overlay District is established to allow continuing use of existing warehousing and light industrial buildings in the Corridor Employment (CE) District and the Corridor Activity Center District (CAC) that were developed for these uses prior to creation of these districts. By allowing these uses to continue, the CLI District protects and promotes owner investment in the existing buildings and site improvements.</t>
+  </si>
+  <si>
+    <t>Transit Oriented Development</t>
+  </si>
+  <si>
+    <t>TOD</t>
+  </si>
+  <si>
+    <t>The TOD District provides for the development and redevelopment of key parcels of land within 3,500 feet of a MARC Station. The TOD District is intended to encourage the development of multi-use centers combining office and high-density residential development that are located and designed for safe and convenient pedestrian access by commuters using the MARC Trains and other public transit links. For sites of least 50 acres, well-designed multi-use centers combining office, high-density residential development with a diversity of dwelling unit types, and retail uses are encouraged. The requirements of this district, in conjunction with the Route 1 Manual and the vehicular and pedestrian improvements that connect internally and with surrounding developments, will result in development that makes use of the commuting potential of the MARC system, creates attractive employment or multi-use centers, and provides for safe and convenient pedestrian travel. Many parcels in the TOD District were developed before this district was created. It is not the intent of these requirements to disallow the continued use of sites developed prior to the TOD District. Additionally, because TOD developments are most effective when comprehensively planned for larger parcels of land surrounding a MARC Station, it is neither the intent of these requirements to encourage smaller, piecemeal TOD developments nor disallow the beneficial use of undeveloped TOD District parcels during the period of time prior to a larger TOD development being assembled. The intent of this district will be achieved by bringing sites into compliance with these requirements and the standards of the Route 1 Manual as a mix of residential and nonresidential uses are redeveloped or expanded. Certain light industrial uses or lower density residential units may also be appropriate with the mix of TOD uses if properly located so as to not overly reduce the available land area for the more dense mix of uses at the core of the TOD development, closer to the MARC Station.</t>
+  </si>
+  <si>
+    <t>Corridor Activity Center</t>
+  </si>
+  <si>
+    <t>CAC</t>
+  </si>
+  <si>
+    <t>The CAC District is intended to provide for the development of pedestrian-oriented, urban activity centers with a mix of uses which may include retail, service, office and residential uses. These centers should be located near to Route 1 and close to residential communities that will benefit from a pedestrian-oriented local business area. The requirements of this district, in conjunction with the Route 1 Manual and the public improvements recommended by the Route 1 Corridor Revitalization Study, vehicular and pedestrian improvements that connect internally and with surrounding developments will result in development that will strengthen nearby communities, provide for safe and convenient pedestrian travel, and improve the streetscape of Route 1 and intersecting roads. Many parcels in the CAC District were developed before this district was created. It is not the intent of these requirements to disallow the continued use of sites developed prior to the CAC District. The intent of this district will be achieved by bringing the sites into compliance with these requirements and the standards of the Route 1 Manual as uses are expanded or redeveloped.</t>
+  </si>
+  <si>
+    <t>Traditional Neighborhood Center</t>
+  </si>
+  <si>
+    <t>TNC</t>
+  </si>
+  <si>
+    <t>The TNC District is intended to provide for the development of pedestrian-oriented, urban activity centers with a mix of retail, service, office and residential uses. These centers should be located near Route 40 and close to residential communities that will benefit from a pedestrian-oriented local business area. The requirements of this district, in conjunction with the Route 40 Manual and the public improvements recommended by the Route 40 Enhancement Study, will result in development that will strengthen nearby communities, provide for safe and convenient pedestrian travel, and improve the streetscape of Route 40 and intersecting roads. Sites within the TNC Overlay may continue to be used, developed and redeveloped in accordance with the underlying zoning. The intent of this district is to provide an alternative method of development for property owners who choose to comply with the Route 40 Manual and the requirements of this district. Development complying with the TNC District requirements will be permitted to include residential development and will have greater flexibility in some bulk requirements.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -953,6 +1260,12 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF313335"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -974,7 +1287,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -982,6 +1295,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2635,4 +2949,538 @@
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{464F2D48-DB33-4D34-8FC3-5B3A744A185C}">
+  <dimension ref="A1:D37"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="40.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" customWidth="1"/>
+    <col min="3" max="3" width="44.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="255.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>229</v>
+      </c>
+      <c r="B2" t="s">
+        <v>123</v>
+      </c>
+      <c r="C2" t="s">
+        <v>230</v>
+      </c>
+      <c r="D2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>232</v>
+      </c>
+      <c r="B3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D3" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>234</v>
+      </c>
+      <c r="B4" t="s">
+        <v>235</v>
+      </c>
+      <c r="C4" t="s">
+        <v>230</v>
+      </c>
+      <c r="D4" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>237</v>
+      </c>
+      <c r="B5" t="s">
+        <v>238</v>
+      </c>
+      <c r="C5" t="s">
+        <v>230</v>
+      </c>
+      <c r="D5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>240</v>
+      </c>
+      <c r="B6" t="s">
+        <v>162</v>
+      </c>
+      <c r="C6" t="s">
+        <v>230</v>
+      </c>
+      <c r="D6" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>240</v>
+      </c>
+      <c r="B7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" t="s">
+        <v>230</v>
+      </c>
+      <c r="D7" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>244</v>
+      </c>
+      <c r="B8" t="s">
+        <v>243</v>
+      </c>
+      <c r="C8" t="s">
+        <v>230</v>
+      </c>
+      <c r="D8" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>247</v>
+      </c>
+      <c r="B9" t="s">
+        <v>246</v>
+      </c>
+      <c r="C9" t="s">
+        <v>230</v>
+      </c>
+      <c r="D9" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>249</v>
+      </c>
+      <c r="B10" t="s">
+        <v>250</v>
+      </c>
+      <c r="C10" t="s">
+        <v>230</v>
+      </c>
+      <c r="D10" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>253</v>
+      </c>
+      <c r="B11" t="s">
+        <v>252</v>
+      </c>
+      <c r="C11" t="s">
+        <v>230</v>
+      </c>
+      <c r="D11" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>256</v>
+      </c>
+      <c r="B12" t="s">
+        <v>255</v>
+      </c>
+      <c r="C12" t="s">
+        <v>230</v>
+      </c>
+      <c r="D12" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>258</v>
+      </c>
+      <c r="B13" t="s">
+        <v>259</v>
+      </c>
+      <c r="C13" t="s">
+        <v>230</v>
+      </c>
+      <c r="D13" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>261</v>
+      </c>
+      <c r="B14" t="s">
+        <v>262</v>
+      </c>
+      <c r="C14" t="s">
+        <v>230</v>
+      </c>
+      <c r="D14" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>264</v>
+      </c>
+      <c r="B15" t="s">
+        <v>265</v>
+      </c>
+      <c r="C15" t="s">
+        <v>230</v>
+      </c>
+      <c r="D15" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>267</v>
+      </c>
+      <c r="B16" t="s">
+        <v>268</v>
+      </c>
+      <c r="C16" t="s">
+        <v>230</v>
+      </c>
+      <c r="D16" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>270</v>
+      </c>
+      <c r="B17" t="s">
+        <v>271</v>
+      </c>
+      <c r="C17" t="s">
+        <v>230</v>
+      </c>
+      <c r="D17" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>273</v>
+      </c>
+      <c r="B18" t="s">
+        <v>274</v>
+      </c>
+      <c r="C18" t="s">
+        <v>230</v>
+      </c>
+      <c r="D18" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>276</v>
+      </c>
+      <c r="B19" t="s">
+        <v>277</v>
+      </c>
+      <c r="C19" t="s">
+        <v>230</v>
+      </c>
+      <c r="D19" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>279</v>
+      </c>
+      <c r="B20" t="s">
+        <v>280</v>
+      </c>
+      <c r="C20" t="s">
+        <v>230</v>
+      </c>
+      <c r="D20" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B21" t="s">
+        <v>283</v>
+      </c>
+      <c r="C21" t="s">
+        <v>230</v>
+      </c>
+      <c r="D21" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>286</v>
+      </c>
+      <c r="B22" t="s">
+        <v>285</v>
+      </c>
+      <c r="C22" t="s">
+        <v>230</v>
+      </c>
+      <c r="D22" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>288</v>
+      </c>
+      <c r="B23" t="s">
+        <v>222</v>
+      </c>
+      <c r="C23" t="s">
+        <v>230</v>
+      </c>
+      <c r="D23" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>292</v>
+      </c>
+      <c r="B24" t="s">
+        <v>290</v>
+      </c>
+      <c r="C24" t="s">
+        <v>230</v>
+      </c>
+      <c r="D24" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>293</v>
+      </c>
+      <c r="B25" t="s">
+        <v>294</v>
+      </c>
+      <c r="C25" t="s">
+        <v>230</v>
+      </c>
+      <c r="D25" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>296</v>
+      </c>
+      <c r="B26" t="s">
+        <v>297</v>
+      </c>
+      <c r="C26" t="s">
+        <v>230</v>
+      </c>
+      <c r="D26" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>299</v>
+      </c>
+      <c r="B27" t="s">
+        <v>300</v>
+      </c>
+      <c r="C27" t="s">
+        <v>230</v>
+      </c>
+      <c r="D27" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>302</v>
+      </c>
+      <c r="B28" t="s">
+        <v>303</v>
+      </c>
+      <c r="C28" t="s">
+        <v>230</v>
+      </c>
+      <c r="D28" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>305</v>
+      </c>
+      <c r="B29" t="s">
+        <v>306</v>
+      </c>
+      <c r="C29" t="s">
+        <v>230</v>
+      </c>
+      <c r="D29" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>308</v>
+      </c>
+      <c r="B30" t="s">
+        <v>309</v>
+      </c>
+      <c r="C30" t="s">
+        <v>230</v>
+      </c>
+      <c r="D30" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>311</v>
+      </c>
+      <c r="B31" t="s">
+        <v>312</v>
+      </c>
+      <c r="C31" t="s">
+        <v>230</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>314</v>
+      </c>
+      <c r="B32" t="s">
+        <v>315</v>
+      </c>
+      <c r="C32" t="s">
+        <v>230</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>317</v>
+      </c>
+      <c r="B33" t="s">
+        <v>297</v>
+      </c>
+      <c r="C33" t="s">
+        <v>230</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>319</v>
+      </c>
+      <c r="B34" t="s">
+        <v>320</v>
+      </c>
+      <c r="C34" t="s">
+        <v>230</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>322</v>
+      </c>
+      <c r="B35" t="s">
+        <v>323</v>
+      </c>
+      <c r="C35" t="s">
+        <v>230</v>
+      </c>
+      <c r="D35" s="5" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>325</v>
+      </c>
+      <c r="B36" t="s">
+        <v>326</v>
+      </c>
+      <c r="C36" t="s">
+        <v>230</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>328</v>
+      </c>
+      <c r="B37" t="s">
+        <v>329</v>
+      </c>
+      <c r="C37" t="s">
+        <v>230</v>
+      </c>
+      <c r="D37" s="5" t="s">
+        <v>330</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>